<commit_message>
Add LK (Leveaniemi-Kiruna) ore combination to forecast model
</commit_message>
<xml_diff>
--- a/forecast_results.xlsx
+++ b/forecast_results.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="38">
   <si>
     <t>Year</t>
   </si>
@@ -98,6 +98,18 @@
     <t>MC perturbation %</t>
   </si>
   <si>
+    <t>LK leach rate (kg/Mton)</t>
+  </si>
+  <si>
+    <t>LK prod winter (Mton)</t>
+  </si>
+  <si>
+    <t>LK prod summer (Mton)</t>
+  </si>
+  <si>
+    <t>LK assumption</t>
+  </si>
+  <si>
     <t>Cu</t>
   </si>
   <si>
@@ -114,6 +126,9 @@
   </si>
   <si>
     <t>mg/L</t>
+  </si>
+  <si>
+    <t>50/50 Leveaniemi+Kiruna (PLACEHOLDER)</t>
   </si>
   <si>
     <t>Cross-Validation Diagnostics -- Random Forest Models</t>
@@ -534,13 +549,13 @@
         <v>6</v>
       </c>
       <c r="C4" s="3">
-        <v>1.086237053972512</v>
+        <v>1.082104974523516</v>
       </c>
       <c r="D4" s="3">
-        <v>1.086237053972512</v>
+        <v>1.082104974523516</v>
       </c>
       <c r="E4" s="3">
-        <v>1.086237053972512</v>
+        <v>1.082104974523516</v>
       </c>
       <c r="F4" s="3">
         <v>1</v>
@@ -554,13 +569,13 @@
         <v>7</v>
       </c>
       <c r="C5" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="D5" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="E5" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="F5" s="3">
         <v>9.567878827961081</v>
@@ -574,13 +589,13 @@
         <v>6</v>
       </c>
       <c r="C6" s="3">
-        <v>1.261430327462896</v>
+        <v>1.109885629409148</v>
       </c>
       <c r="D6" s="3">
-        <v>1.261430327462896</v>
+        <v>1.109885629409148</v>
       </c>
       <c r="E6" s="3">
-        <v>1.261430327462896</v>
+        <v>1.109885629409148</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
@@ -594,13 +609,13 @@
         <v>7</v>
       </c>
       <c r="C7" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="D7" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="E7" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="F7" s="3">
         <v>9.133794571254251</v>
@@ -614,13 +629,13 @@
         <v>6</v>
       </c>
       <c r="C8" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="D8" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="E8" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
@@ -634,13 +649,13 @@
         <v>7</v>
       </c>
       <c r="C9" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="D9" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="E9" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="F9" s="3">
         <v>8.74101759041824</v>
@@ -654,13 +669,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="D10" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="E10" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="F10" s="3">
         <v>1</v>
@@ -674,13 +689,13 @@
         <v>7</v>
       </c>
       <c r="C11" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="D11" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="E11" s="3">
-        <v>11.6343130934851</v>
+        <v>11.58623887058581</v>
       </c>
       <c r="F11" s="3">
         <v>8.383919507897639</v>
@@ -694,13 +709,13 @@
         <v>6</v>
       </c>
       <c r="C12" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="D12" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="E12" s="3">
-        <v>1.261430327462896</v>
+        <v>1.097521415993899</v>
       </c>
       <c r="F12" s="3">
         <v>1</v>
@@ -753,13 +768,13 @@
         <v>6</v>
       </c>
       <c r="C4" s="3">
-        <v>0.02911477131449258</v>
+        <v>0.02491116891813362</v>
       </c>
       <c r="D4" s="3">
-        <v>0.02911477131449259</v>
+        <v>0.02491116891813363</v>
       </c>
       <c r="E4" s="3">
-        <v>0.0291147713144926</v>
+        <v>0.02491116891813364</v>
       </c>
       <c r="F4" s="3">
         <v>0.01</v>
@@ -773,13 +788,13 @@
         <v>6</v>
       </c>
       <c r="C5" s="3">
-        <v>1.706596593546433</v>
+        <v>1.613042108765848</v>
       </c>
       <c r="D5" s="3">
-        <v>1.706596593546434</v>
+        <v>1.613042108765849</v>
       </c>
       <c r="E5" s="3">
-        <v>1.912915602358276</v>
+        <v>1.785579221640004</v>
       </c>
       <c r="F5" s="3">
         <v>1.523978999244271</v>
@@ -793,13 +808,13 @@
         <v>6</v>
       </c>
       <c r="C6" s="3">
-        <v>0.3907724212133894</v>
+        <v>0.4544787355202886</v>
       </c>
       <c r="D6" s="3">
-        <v>0.3907724212133897</v>
+        <v>0.4544787355202888</v>
       </c>
       <c r="E6" s="3">
-        <v>0.39077242121339</v>
+        <v>0.4544787355202891</v>
       </c>
       <c r="F6" s="3">
         <v>0.01</v>
@@ -813,13 +828,13 @@
         <v>6</v>
       </c>
       <c r="C7" s="3">
-        <v>1.706596593546433</v>
+        <v>1.613042108765848</v>
       </c>
       <c r="D7" s="3">
-        <v>1.706596593546434</v>
+        <v>1.613042108765849</v>
       </c>
       <c r="E7" s="3">
-        <v>1.912915602358275</v>
+        <v>1.785579221640004</v>
       </c>
       <c r="F7" s="3">
         <v>1.447846488956811</v>
@@ -833,13 +848,13 @@
         <v>6</v>
       </c>
       <c r="C8" s="3">
-        <v>0.3900324769413433</v>
+        <v>0.4530883062439007</v>
       </c>
       <c r="D8" s="3">
-        <v>0.3900324769413436</v>
+        <v>0.4530883062439008</v>
       </c>
       <c r="E8" s="3">
-        <v>0.3900324769413439</v>
+        <v>0.4530883062439011</v>
       </c>
       <c r="F8" s="3">
         <v>0.01</v>
@@ -853,13 +868,13 @@
         <v>6</v>
       </c>
       <c r="C9" s="3">
-        <v>1.706596593546433</v>
+        <v>1.613042108765848</v>
       </c>
       <c r="D9" s="3">
-        <v>1.706596593546434</v>
+        <v>1.613042108765849</v>
       </c>
       <c r="E9" s="3">
-        <v>1.912915602358276</v>
+        <v>1.785579221640004</v>
       </c>
       <c r="F9" s="3">
         <v>1.378958716428422</v>
@@ -873,13 +888,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="3">
-        <v>0.3851773976897397</v>
+        <v>0.4508862956636594</v>
       </c>
       <c r="D10" s="3">
-        <v>0.38517739768974</v>
+        <v>0.4508862956636596</v>
       </c>
       <c r="E10" s="3">
-        <v>0.3851773976897402</v>
+        <v>0.4508862956636598</v>
       </c>
       <c r="F10" s="3">
         <v>0.01</v>
@@ -893,13 +908,13 @@
         <v>6</v>
       </c>
       <c r="C11" s="3">
-        <v>1.706596593546433</v>
+        <v>1.613042108765848</v>
       </c>
       <c r="D11" s="3">
-        <v>1.706596593546434</v>
+        <v>1.613042108765849</v>
       </c>
       <c r="E11" s="3">
-        <v>1.912915602358276</v>
+        <v>1.785579221640004</v>
       </c>
       <c r="F11" s="3">
         <v>1.316328540325322</v>
@@ -913,13 +928,13 @@
         <v>6</v>
       </c>
       <c r="C12" s="3">
-        <v>0.3851773976897397</v>
+        <v>0.4508862956636595</v>
       </c>
       <c r="D12" s="3">
-        <v>0.38517739768974</v>
+        <v>0.4508862956636597</v>
       </c>
       <c r="E12" s="3">
-        <v>0.3851773976897402</v>
+        <v>0.4508862956636599</v>
       </c>
       <c r="F12" s="3">
         <v>0.01</v>
@@ -972,13 +987,13 @@
         <v>6</v>
       </c>
       <c r="C4" s="3">
-        <v>2.831359765716891</v>
+        <v>3.100228386527359</v>
       </c>
       <c r="D4" s="3">
-        <v>2.831359765716893</v>
+        <v>3.10022838652736</v>
       </c>
       <c r="E4" s="3">
-        <v>2.831359765716893</v>
+        <v>3.100228386527361</v>
       </c>
       <c r="F4" s="3">
         <v>1.88</v>
@@ -992,13 +1007,13 @@
         <v>6</v>
       </c>
       <c r="C5" s="3">
-        <v>18.01214270230315</v>
+        <v>17.7513965627652</v>
       </c>
       <c r="D5" s="3">
-        <v>18.01214270230316</v>
+        <v>17.75139656276521</v>
       </c>
       <c r="E5" s="3">
-        <v>19.54907362386195</v>
+        <v>18.80206222272055</v>
       </c>
       <c r="F5" s="3">
         <v>15.08804349264114</v>
@@ -1012,13 +1027,13 @@
         <v>6</v>
       </c>
       <c r="C6" s="3">
-        <v>2.964979334975452</v>
+        <v>3.181577512249138</v>
       </c>
       <c r="D6" s="3">
-        <v>2.964979334975454</v>
+        <v>3.181577512249139</v>
       </c>
       <c r="E6" s="3">
-        <v>2.964979334975454</v>
+        <v>3.18157751224914</v>
       </c>
       <c r="F6" s="3">
         <v>1.88</v>
@@ -1032,13 +1047,13 @@
         <v>6</v>
       </c>
       <c r="C7" s="3">
-        <v>18.01214270230315</v>
+        <v>17.7513965627652</v>
       </c>
       <c r="D7" s="3">
-        <v>18.01214270230316</v>
+        <v>17.75139656276521</v>
       </c>
       <c r="E7" s="3">
-        <v>19.54907362386195</v>
+        <v>18.80206222272055</v>
       </c>
       <c r="F7" s="3">
         <v>14.57073642007869</v>
@@ -1052,13 +1067,13 @@
         <v>6</v>
       </c>
       <c r="C8" s="3">
-        <v>2.960321303452078</v>
+        <v>3.160465966063362</v>
       </c>
       <c r="D8" s="3">
-        <v>2.960321303452079</v>
+        <v>3.160465966063363</v>
       </c>
       <c r="E8" s="3">
-        <v>2.96032130345208</v>
+        <v>3.160465966063365</v>
       </c>
       <c r="F8" s="3">
         <v>1.88</v>
@@ -1072,13 +1087,13 @@
         <v>6</v>
       </c>
       <c r="C9" s="3">
-        <v>18.01214270230315</v>
+        <v>17.7513965627652</v>
       </c>
       <c r="D9" s="3">
-        <v>18.01214270230316</v>
+        <v>17.75139656276521</v>
       </c>
       <c r="E9" s="3">
-        <v>19.54907362386195</v>
+        <v>18.80206222272055</v>
       </c>
       <c r="F9" s="3">
         <v>14.09653655111274</v>
@@ -1092,13 +1107,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="3">
-        <v>2.978965942571358</v>
+        <v>3.144094756525073</v>
       </c>
       <c r="D10" s="3">
-        <v>2.978965942571359</v>
+        <v>3.144094756525074</v>
       </c>
       <c r="E10" s="3">
-        <v>2.97896594257136</v>
+        <v>3.144094756525075</v>
       </c>
       <c r="F10" s="3">
         <v>1.88</v>
@@ -1112,13 +1127,13 @@
         <v>6</v>
       </c>
       <c r="C11" s="3">
-        <v>18.01214270230315</v>
+        <v>17.7513965627652</v>
       </c>
       <c r="D11" s="3">
-        <v>18.01214270230316</v>
+        <v>17.75139656276521</v>
       </c>
       <c r="E11" s="3">
-        <v>19.54907362386195</v>
+        <v>18.80206222272055</v>
       </c>
       <c r="F11" s="3">
         <v>13.66027121934641</v>
@@ -1132,13 +1147,13 @@
         <v>6</v>
       </c>
       <c r="C12" s="3">
-        <v>2.95796359298687</v>
+        <v>3.155430275700878</v>
       </c>
       <c r="D12" s="3">
-        <v>2.957963592986871</v>
+        <v>3.155430275700879</v>
       </c>
       <c r="E12" s="3">
-        <v>2.957963592986871</v>
+        <v>3.155430275700881</v>
       </c>
       <c r="F12" s="3">
         <v>1.88</v>
@@ -1191,13 +1206,13 @@
         <v>6</v>
       </c>
       <c r="C4" s="3">
-        <v>0.009014615730679918</v>
+        <v>0.01587708661975399</v>
       </c>
       <c r="D4" s="3">
-        <v>0.009014615730679919</v>
+        <v>0.01587708661975399</v>
       </c>
       <c r="E4" s="3">
-        <v>0.009014615730679923</v>
+        <v>0.01587708661975399</v>
       </c>
       <c r="F4" s="3">
         <v>0.0003330046440613271</v>
@@ -1211,13 +1226,13 @@
         <v>7</v>
       </c>
       <c r="C5" s="3">
-        <v>0.7997456999827068</v>
+        <v>0.7917714612731978</v>
       </c>
       <c r="D5" s="3">
-        <v>0.7997456999827069</v>
+        <v>0.791771461273198</v>
       </c>
       <c r="E5" s="3">
-        <v>0.7997456999827071</v>
+        <v>0.7917714612731981</v>
       </c>
       <c r="F5" s="3">
         <v>0.6972848654290419</v>
@@ -1231,13 +1246,13 @@
         <v>6</v>
       </c>
       <c r="C6" s="3">
-        <v>0.0397754259161901</v>
+        <v>0.05559533671785844</v>
       </c>
       <c r="D6" s="3">
-        <v>0.03977542591619011</v>
+        <v>0.05559533671785846</v>
       </c>
       <c r="E6" s="3">
-        <v>0.03977542591619012</v>
+        <v>0.05559533671785848</v>
       </c>
       <c r="F6" s="3">
         <v>0.0003350082221816188</v>
@@ -1251,13 +1266,13 @@
         <v>7</v>
       </c>
       <c r="C7" s="3">
-        <v>0.7997456999827068</v>
+        <v>0.7917714612731978</v>
       </c>
       <c r="D7" s="3">
-        <v>0.7997456999827069</v>
+        <v>0.791771461273198</v>
       </c>
       <c r="E7" s="3">
-        <v>0.7997456999827071</v>
+        <v>0.7917714612731981</v>
       </c>
       <c r="F7" s="3">
         <v>0.6702250485979465</v>
@@ -1271,13 +1286,13 @@
         <v>6</v>
       </c>
       <c r="C8" s="3">
-        <v>0.0397754259161901</v>
+        <v>0.05555969749044021</v>
       </c>
       <c r="D8" s="3">
-        <v>0.03977542591619011</v>
+        <v>0.05555969749044023</v>
       </c>
       <c r="E8" s="3">
-        <v>0.03977542591619012</v>
+        <v>0.05555969749044024</v>
       </c>
       <c r="F8" s="3">
         <v>0.0003368479467258601</v>
@@ -1291,13 +1306,13 @@
         <v>7</v>
       </c>
       <c r="C9" s="3">
-        <v>0.7997456999827068</v>
+        <v>0.7917714612731978</v>
       </c>
       <c r="D9" s="3">
-        <v>0.7997456999827069</v>
+        <v>0.791771461273198</v>
       </c>
       <c r="E9" s="3">
-        <v>0.7997456999827071</v>
+        <v>0.7917714612731981</v>
       </c>
       <c r="F9" s="3">
         <v>0.6454201265774787</v>
@@ -1311,13 +1326,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="3">
-        <v>0.03823213418886595</v>
+        <v>0.05523441532185528</v>
       </c>
       <c r="D10" s="3">
-        <v>0.03823213418886597</v>
+        <v>0.05523441532185529</v>
       </c>
       <c r="E10" s="3">
-        <v>0.03823213418886597</v>
+        <v>0.05523441532185531</v>
       </c>
       <c r="F10" s="3">
         <v>0.0003385431281216679</v>
@@ -1331,13 +1346,13 @@
         <v>7</v>
       </c>
       <c r="C11" s="3">
-        <v>0.7997456999827068</v>
+        <v>0.7917714612731978</v>
       </c>
       <c r="D11" s="3">
-        <v>0.7997456999827069</v>
+        <v>0.791771461273198</v>
       </c>
       <c r="E11" s="3">
-        <v>0.7997456999827071</v>
+        <v>0.7917714612731981</v>
       </c>
       <c r="F11" s="3">
         <v>0.622599522349361</v>
@@ -1351,13 +1366,13 @@
         <v>6</v>
       </c>
       <c r="C12" s="3">
-        <v>0.03823213418886595</v>
+        <v>0.05523441532185528</v>
       </c>
       <c r="D12" s="3">
-        <v>0.03823213418886597</v>
+        <v>0.05523441532185529</v>
       </c>
       <c r="E12" s="3">
-        <v>0.03823213418886597</v>
+        <v>0.05523441532185531</v>
       </c>
       <c r="F12" s="3">
         <v>0.0003401101571359144</v>
@@ -1370,19 +1385,22 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="9" width="18.7109375" customWidth="1"/>
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="11" max="11" width="26.7109375" customWidth="1"/>
+    <col min="12" max="13" width="24.7109375" customWidth="1"/>
+    <col min="14" max="14" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -1413,13 +1431,25 @@
       <c r="J3" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C4">
         <v>22</v>
@@ -1428,13 +1458,13 @@
         <v>9</v>
       </c>
       <c r="E4">
-        <v>0.7645999999999999</v>
+        <v>0.7577</v>
       </c>
       <c r="F4">
-        <v>0.0053</v>
+        <v>0.0233</v>
       </c>
       <c r="G4">
-        <v>0.9716</v>
+        <v>0.9744</v>
       </c>
       <c r="H4">
         <v>4</v>
@@ -1445,13 +1475,25 @@
       <c r="J4">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4">
+        <v>6.513</v>
+      </c>
+      <c r="L4">
+        <v>1.6667</v>
+      </c>
+      <c r="M4">
+        <v>2.5667</v>
+      </c>
+      <c r="N4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C5">
         <v>22</v>
@@ -1460,13 +1502,13 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>0.7799</v>
+        <v>0.7691</v>
       </c>
       <c r="F5">
-        <v>0.0187</v>
+        <v>0.0291</v>
       </c>
       <c r="G5">
-        <v>0.9656</v>
+        <v>0.9701</v>
       </c>
       <c r="H5">
         <v>4</v>
@@ -1477,13 +1519,25 @@
       <c r="J5">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5">
+        <v>1523.65</v>
+      </c>
+      <c r="L5">
+        <v>1.6667</v>
+      </c>
+      <c r="M5">
+        <v>2.5667</v>
+      </c>
+      <c r="N5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C6">
         <v>22</v>
@@ -1492,13 +1546,13 @@
         <v>9</v>
       </c>
       <c r="E6">
-        <v>0.8563</v>
+        <v>0.8431999999999999</v>
       </c>
       <c r="F6">
-        <v>0.0305</v>
+        <v>0.0328</v>
       </c>
       <c r="G6">
-        <v>0.9728</v>
+        <v>0.9766</v>
       </c>
       <c r="H6">
         <v>4</v>
@@ -1509,13 +1563,25 @@
       <c r="J6">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="K6">
+        <v>219925</v>
+      </c>
+      <c r="L6">
+        <v>1.6667</v>
+      </c>
+      <c r="M6">
+        <v>2.5667</v>
+      </c>
+      <c r="N6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>22</v>
@@ -1524,13 +1590,13 @@
         <v>9</v>
       </c>
       <c r="E7">
-        <v>0.8566</v>
+        <v>0.8537</v>
       </c>
       <c r="F7">
-        <v>0.045</v>
+        <v>0.0507</v>
       </c>
       <c r="G7">
-        <v>0.9733000000000001</v>
+        <v>0.9723000000000001</v>
       </c>
       <c r="H7">
         <v>4</v>
@@ -1540,6 +1606,18 @@
       </c>
       <c r="J7">
         <v>15</v>
+      </c>
+      <c r="K7">
+        <v>0.9025</v>
+      </c>
+      <c r="L7">
+        <v>1.6667</v>
+      </c>
+      <c r="M7">
+        <v>2.5667</v>
+      </c>
+      <c r="N7" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>